<commit_message>
Log Sep 27 inventory counts (pharmacies 3 and 31), review pending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -2140,7 +2140,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="B8" s="5">
         <f>IF(A8="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A8,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2149,10 +2153,20 @@
         <f>IF(A8="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A8,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
+      <c r="D8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="5">
         <f>IF(E8="","",IF(AND(F8="نعم",G8="نعم"),"جرد + مراجعة",IF(F8="نعم","جرد فقط",IF(G8="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2163,7 +2177,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="B9" s="5">
         <f>IF(A9="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A9,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2172,10 +2190,20 @@
         <f>IF(A9="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A9,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
+      <c r="D9" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="5">
         <f>IF(E9="","",IF(AND(F9="نعم",G9="نعم"),"جرد + مراجعة",IF(F9="نعم","جرد فقط",IF(G9="نعم","مراجعة فقط",""))))</f>
         <v/>

</xml_diff>

<commit_message>
Log Sep 27 reviews for pharmacies 3 and 31
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -2166,7 +2166,11 @@
           <t>نعم</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H8" s="5">
         <f>IF(E8="","",IF(AND(F8="نعم",G8="نعم"),"جرد + مراجعة",IF(F8="نعم","جرد فقط",IF(G8="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2191,65 +2195,97 @@
         <v/>
       </c>
       <c r="D9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H9" s="5">
+        <f>IF(E9="","",IF(AND(F9="نعم",G9="نعم"),"جرد + مراجعة",IF(F9="نعم","جرد فقط",IF(G9="نعم","مراجعة فقط",""))))</f>
+        <v/>
+      </c>
+      <c r="I9" s="9">
+        <f>IF(H9="جرد + مراجعة",الإعدادات!$B$2,IF(H9="مراجعة فقط",الإعدادات!$B$3,IF(H9="جرد فقط",الإعدادات!$B$4,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B10" s="5">
+        <f>IF(A10="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A10,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>IF(A10="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A10,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H10" s="5">
+        <f>IF(E10="","",IF(AND(F10="نعم",G10="نعم"),"جرد + مراجعة",IF(F10="نعم","جرد فقط",IF(G10="نعم","مراجعة فقط",""))))</f>
+        <v/>
+      </c>
+      <c r="I10" s="9">
+        <f>IF(H10="جرد + مراجعة",الإعدادات!$B$2,IF(H10="مراجعة فقط",الإعدادات!$B$3,IF(H10="جرد فقط",الإعدادات!$B$4,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>IF(A11="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A11,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>IF(A11="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A11,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D11" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>د. علي خليفة</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="5">
-        <f>IF(E9="","",IF(AND(F9="نعم",G9="نعم"),"جرد + مراجعة",IF(F9="نعم","جرد فقط",IF(G9="نعم","مراجعة فقط",""))))</f>
-        <v/>
-      </c>
-      <c r="I9" s="9">
-        <f>IF(H9="جرد + مراجعة",الإعدادات!$B$2,IF(H9="مراجعة فقط",الإعدادات!$B$3,IF(H9="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="5">
-        <f>IF(A10="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A10,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="C10" s="5">
-        <f>IF(A10="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A10,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="5">
-        <f>IF(E10="","",IF(AND(F10="نعم",G10="نعم"),"جرد + مراجعة",IF(F10="نعم","جرد فقط",IF(G10="نعم","مراجعة فقط",""))))</f>
-        <v/>
-      </c>
-      <c r="I10" s="9">
-        <f>IF(H10="جرد + مراجعة",الإعدادات!$B$2,IF(H10="مراجعة فقط",الإعدادات!$B$3,IF(H10="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="5">
-        <f>IF(A11="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A11,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="C11" s="5">
-        <f>IF(A11="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A11,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H11" s="5">
         <f>IF(E11="","",IF(AND(F11="نعم",G11="نعم"),"جرد + مراجعة",IF(F11="نعم","جرد فقط",IF(G11="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2260,7 +2296,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="B12" s="5">
         <f>IF(A12="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A12,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2269,10 +2309,20 @@
         <f>IF(A12="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A12,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
+      <c r="D12" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H12" s="5">
         <f>IF(E12="","",IF(AND(F12="نعم",G12="نعم"),"جرد + مراجعة",IF(F12="نعم","جرد فقط",IF(G12="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2283,7 +2333,11 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="B13" s="5">
         <f>IF(A13="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A13,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2292,10 +2346,20 @@
         <f>IF(A13="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A13,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
+      <c r="D13" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H13" s="5">
         <f>IF(E13="","",IF(AND(F13="نعم",G13="نعم"),"جرد + مراجعة",IF(F13="نعم","جرد فقط",IF(G13="نعم","مراجعة فقط",""))))</f>
         <v/>

</xml_diff>

<commit_message>
Add Ayman Hussein review (pharmacy 31) and Sep 28 counts (29, 22)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -658,7 +658,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
       <c r="B7" s="5">
         <f>IF(A7="","",COUNTIFS(السجل!$E$2:$E$1000,A7,السجل!$H$2:$H$1000,"جرد + مراجعة"))</f>
         <v/>
@@ -2370,7 +2374,11 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n"/>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="B14" s="5">
         <f>IF(A14="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A14,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2379,10 +2387,20 @@
         <f>IF(A14="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A14,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
+      <c r="D14" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H14" s="5">
         <f>IF(E14="","",IF(AND(F14="نعم",G14="نعم"),"جرد + مراجعة",IF(F14="نعم","جرد فقط",IF(G14="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2393,7 +2411,11 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="B15" s="5">
         <f>IF(A15="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A15,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2402,10 +2424,20 @@
         <f>IF(A15="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A15,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
+      <c r="D15" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="5">
         <f>IF(E15="","",IF(AND(F15="نعم",G15="نعم"),"جرد + مراجعة",IF(F15="نعم","جرد فقط",IF(G15="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2416,7 +2448,11 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="B16" s="5">
         <f>IF(A16="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A16,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2425,10 +2461,20 @@
         <f>IF(A16="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A16,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
+      <c r="D16" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="5">
         <f>IF(E16="","",IF(AND(F16="نعم",G16="نعم"),"جرد + مراجعة",IF(F16="نعم","جرد فقط",IF(G16="نعم","مراجعة فقط",""))))</f>
         <v/>

</xml_diff>

<commit_message>
Log Sep 28 reviews for pharmacies 29 and 22
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -2437,7 +2437,11 @@
           <t>نعم</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H15" s="5">
         <f>IF(E15="","",IF(AND(F15="نعم",G15="نعم"),"جرد + مراجعة",IF(F15="نعم","جرد فقط",IF(G15="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2462,88 +2466,134 @@
         <v/>
       </c>
       <c r="D16" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H16" s="5">
+        <f>IF(E16="","",IF(AND(F16="نعم",G16="نعم"),"جرد + مراجعة",IF(F16="نعم","جرد فقط",IF(G16="نعم","مراجعة فقط",""))))</f>
+        <v/>
+      </c>
+      <c r="I16" s="9">
+        <f>IF(H16="جرد + مراجعة",الإعدادات!$B$2,IF(H16="مراجعة فقط",الإعدادات!$B$3,IF(H16="جرد فقط",الإعدادات!$B$4,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>IF(A17="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A17,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C17" s="5">
+        <f>IF(A17="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A17,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H17" s="5">
+        <f>IF(E17="","",IF(AND(F17="نعم",G17="نعم"),"جرد + مراجعة",IF(F17="نعم","جرد فقط",IF(G17="نعم","مراجعة فقط",""))))</f>
+        <v/>
+      </c>
+      <c r="I17" s="9">
+        <f>IF(H17="جرد + مراجعة",الإعدادات!$B$2,IF(H17="مراجعة فقط",الإعدادات!$B$3,IF(H17="جرد فقط",الإعدادات!$B$4,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>IF(A18="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A18,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f>IF(A18="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A18,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="H18" s="5">
+        <f>IF(E18="","",IF(AND(F18="نعم",G18="نعم"),"جرد + مراجعة",IF(F18="نعم","جرد فقط",IF(G18="نعم","مراجعة فقط",""))))</f>
+        <v/>
+      </c>
+      <c r="I18" s="9">
+        <f>IF(H18="جرد + مراجعة",الإعدادات!$B$2,IF(H18="مراجعة فقط",الإعدادات!$B$3,IF(H18="جرد فقط",الإعدادات!$B$4,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>IF(A19="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A19,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="C19" s="5">
+        <f>IF(A19="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A19,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
+        <v/>
+      </c>
+      <c r="D19" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>د. حسام شلش</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="5">
-        <f>IF(E16="","",IF(AND(F16="نعم",G16="نعم"),"جرد + مراجعة",IF(F16="نعم","جرد فقط",IF(G16="نعم","مراجعة فقط",""))))</f>
-        <v/>
-      </c>
-      <c r="I16" s="9">
-        <f>IF(H16="جرد + مراجعة",الإعدادات!$B$2,IF(H16="مراجعة فقط",الإعدادات!$B$3,IF(H16="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="5">
-        <f>IF(A17="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A17,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="C17" s="5">
-        <f>IF(A17="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A17,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="5">
-        <f>IF(E17="","",IF(AND(F17="نعم",G17="نعم"),"جرد + مراجعة",IF(F17="نعم","جرد فقط",IF(G17="نعم","مراجعة فقط",""))))</f>
-        <v/>
-      </c>
-      <c r="I17" s="9">
-        <f>IF(H17="جرد + مراجعة",الإعدادات!$B$2,IF(H17="مراجعة فقط",الإعدادات!$B$3,IF(H17="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="5">
-        <f>IF(A18="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A18,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="C18" s="5">
-        <f>IF(A18="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A18,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="5">
-        <f>IF(E18="","",IF(AND(F18="نعم",G18="نعم"),"جرد + مراجعة",IF(F18="نعم","جرد فقط",IF(G18="نعم","مراجعة فقط",""))))</f>
-        <v/>
-      </c>
-      <c r="I18" s="9">
-        <f>IF(H18="جرد + مراجعة",الإعدادات!$B$2,IF(H18="مراجعة فقط",الإعدادات!$B$3,IF(H18="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="5">
-        <f>IF(A19="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A19,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="C19" s="5">
-        <f>IF(A19="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A19,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H19" s="5">
         <f>IF(E19="","",IF(AND(F19="نعم",G19="نعم"),"جرد + مراجعة",IF(F19="نعم","جرد فقط",IF(G19="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2554,7 +2604,11 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n"/>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="B20" s="5">
         <f>IF(A20="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A20,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2563,10 +2617,20 @@
         <f>IF(A20="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A20,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
+      <c r="D20" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H20" s="5">
         <f>IF(E20="","",IF(AND(F20="نعم",G20="نعم"),"جرد + مراجعة",IF(F20="نعم","جرد فقط",IF(G20="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2577,7 +2641,11 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n"/>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="B21" s="5">
         <f>IF(A21="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A21,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2586,10 +2654,20 @@
         <f>IF(A21="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A21,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
+      <c r="D21" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H21" s="5">
         <f>IF(E21="","",IF(AND(F21="نعم",G21="نعم"),"جرد + مراجعة",IF(F21="نعم","جرد فقط",IF(G21="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2600,7 +2678,11 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="B22" s="5">
         <f>IF(A22="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A22,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2609,10 +2691,20 @@
         <f>IF(A22="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A22,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
+      <c r="D22" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H22" s="5">
         <f>IF(E22="","",IF(AND(F22="نعم",G22="نعم"),"جرد + مراجعة",IF(F22="نعم","جرد فقط",IF(G22="نعم","مراجعة فقط",""))))</f>
         <v/>

</xml_diff>

<commit_message>
Remove Ayman Hussein from Sep 28 review of pharmacy 22
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -2678,11 +2678,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+      <c r="A22" s="4" t="n"/>
       <c r="B22" s="5">
         <f>IF(A22="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A22,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2691,20 +2687,10 @@
         <f>IF(A22="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A22,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D22" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>د. أيمن حسين</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
       <c r="H22" s="5">
         <f>IF(E22="","",IF(AND(F22="نعم",G22="نعم"),"جرد + مراجعة",IF(F22="نعم","جرد فقط",IF(G22="نعم","مراجعة فقط",""))))</f>
         <v/>

</xml_diff>

<commit_message>
Log Sep 29 counts and reviews (pharmacies 21 and 30)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -685,7 +685,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
       <c r="B8" s="5">
         <f>IF(A8="","",COUNTIFS(السجل!$E$2:$E$1000,A8,السجل!$H$2:$H$1000,"جرد + مراجعة"))</f>
         <v/>
@@ -2678,7 +2682,11 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B22" s="5">
         <f>IF(A22="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A22,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2687,10 +2695,24 @@
         <f>IF(A22="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A22,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
+      <c r="D22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H22" s="5">
         <f>IF(E22="","",IF(AND(F22="نعم",G22="نعم"),"جرد + مراجعة",IF(F22="نعم","جرد فقط",IF(G22="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2701,7 +2723,11 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B23" s="5">
         <f>IF(A23="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A23,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2710,10 +2736,20 @@
         <f>IF(A23="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A23,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
+      <c r="D23" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H23" s="5">
         <f>IF(E23="","",IF(AND(F23="نعم",G23="نعم"),"جرد + مراجعة",IF(F23="نعم","جرد فقط",IF(G23="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2724,7 +2760,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n"/>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B24" s="5">
         <f>IF(A24="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A24,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2733,10 +2773,20 @@
         <f>IF(A24="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A24,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
+      <c r="D24" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H24" s="5">
         <f>IF(E24="","",IF(AND(F24="نعم",G24="نعم"),"جرد + مراجعة",IF(F24="نعم","جرد فقط",IF(G24="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2747,7 +2797,11 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n"/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B25" s="5">
         <f>IF(A25="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A25,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2756,10 +2810,20 @@
         <f>IF(A25="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A25,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
+      <c r="D25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H25" s="5">
         <f>IF(E25="","",IF(AND(F25="نعم",G25="نعم"),"جرد + مراجعة",IF(F25="نعم","جرد فقط",IF(G25="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2770,7 +2834,11 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n"/>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B26" s="5">
         <f>IF(A26="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A26,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2779,10 +2847,20 @@
         <f>IF(A26="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A26,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
+      <c r="D26" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H26" s="5">
         <f>IF(E26="","",IF(AND(F26="نعم",G26="نعم"),"جرد + مراجعة",IF(F26="نعم","جرد فقط",IF(G26="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2793,7 +2871,11 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n"/>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B27" s="5">
         <f>IF(A27="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A27,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2802,10 +2884,24 @@
         <f>IF(A27="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A27,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
+      <c r="D27" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H27" s="5">
         <f>IF(E27="","",IF(AND(F27="نعم",G27="نعم"),"جرد + مراجعة",IF(F27="نعم","جرد فقط",IF(G27="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2816,7 +2912,11 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n"/>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B28" s="5">
         <f>IF(A28="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A28,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2825,10 +2925,20 @@
         <f>IF(A28="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A28,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
+      <c r="D28" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H28" s="5">
         <f>IF(E28="","",IF(AND(F28="نعم",G28="نعم"),"جرد + مراجعة",IF(F28="نعم","جرد فقط",IF(G28="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2839,7 +2949,11 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n"/>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B29" s="5">
         <f>IF(A29="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A29,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2848,10 +2962,20 @@
         <f>IF(A29="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A29,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
+      <c r="D29" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H29" s="5">
         <f>IF(E29="","",IF(AND(F29="نعم",G29="نعم"),"جرد + مراجعة",IF(F29="نعم","جرد فقط",IF(G29="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2862,7 +2986,11 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n"/>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B30" s="5">
         <f>IF(A30="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A30,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2871,10 +2999,20 @@
         <f>IF(A30="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A30,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
-      <c r="G30" s="4" t="n"/>
+      <c r="D30" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H30" s="5">
         <f>IF(E30="","",IF(AND(F30="نعم",G30="نعم"),"جرد + مراجعة",IF(F30="نعم","جرد فقط",IF(G30="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -2885,7 +3023,11 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n"/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="B31" s="5">
         <f>IF(A31="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A31,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -2894,10 +3036,20 @@
         <f>IF(A31="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A31,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
+      <c r="D31" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H31" s="5">
         <f>IF(E31="","",IF(AND(F31="نعم",G31="نعم"),"جرد + مراجعة",IF(F31="نعم","جرد فقط",IF(G31="نعم","مراجعة فقط",""))))</f>
         <v/>

</xml_diff>

<commit_message>
Log Sep 30 counts and reviews (pharmacies 10 and 17)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -3060,7 +3060,11 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n"/>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B32" s="5">
         <f>IF(A32="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A32,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3069,10 +3073,24 @@
         <f>IF(A32="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A32,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
+      <c r="D32" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H32" s="5">
         <f>IF(E32="","",IF(AND(F32="نعم",G32="نعم"),"جرد + مراجعة",IF(F32="نعم","جرد فقط",IF(G32="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -3083,7 +3101,11 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n"/>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B33" s="5">
         <f>IF(A33="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A33,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3092,10 +3114,20 @@
         <f>IF(A33="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A33,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
+      <c r="D33" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H33" s="5">
         <f>IF(E33="","",IF(AND(F33="نعم",G33="نعم"),"جرد + مراجعة",IF(F33="نعم","جرد فقط",IF(G33="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -3106,7 +3138,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n"/>
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B34" s="5">
         <f>IF(A34="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A34,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3115,10 +3151,20 @@
         <f>IF(A34="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A34,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
+      <c r="D34" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H34" s="5">
         <f>IF(E34="","",IF(AND(F34="نعم",G34="نعم"),"جرد + مراجعة",IF(F34="نعم","جرد فقط",IF(G34="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -3129,7 +3175,11 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n"/>
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B35" s="5">
         <f>IF(A35="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A35,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3138,10 +3188,20 @@
         <f>IF(A35="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A35,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
-      <c r="G35" s="4" t="n"/>
+      <c r="D35" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H35" s="5">
         <f>IF(E35="","",IF(AND(F35="نعم",G35="نعم"),"جرد + مراجعة",IF(F35="نعم","جرد فقط",IF(G35="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -3152,7 +3212,11 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n"/>
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B36" s="5">
         <f>IF(A36="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A36,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3161,10 +3225,24 @@
         <f>IF(A36="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A36,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
+      <c r="D36" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H36" s="5">
         <f>IF(E36="","",IF(AND(F36="نعم",G36="نعم"),"جرد + مراجعة",IF(F36="نعم","جرد فقط",IF(G36="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -3175,7 +3253,11 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n"/>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B37" s="5">
         <f>IF(A37="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A37,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3184,10 +3266,20 @@
         <f>IF(A37="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A37,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
+      <c r="D37" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H37" s="5">
         <f>IF(E37="","",IF(AND(F37="نعم",G37="نعم"),"جرد + مراجعة",IF(F37="نعم","جرد فقط",IF(G37="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -3198,7 +3290,11 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n"/>
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B38" s="5">
         <f>IF(A38="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A38,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3207,10 +3303,20 @@
         <f>IF(A38="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A38,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
+      <c r="D38" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H38" s="5">
         <f>IF(E38="","",IF(AND(F38="نعم",G38="نعم"),"جرد + مراجعة",IF(F38="نعم","جرد فقط",IF(G38="نعم","مراجعة فقط",""))))</f>
         <v/>
@@ -3221,7 +3327,11 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n"/>
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B39" s="5">
         <f>IF(A39="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A39,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3230,10 +3340,20 @@
         <f>IF(A39="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A39,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
+      <c r="D39" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H39" s="5">
         <f>IF(E39="","",IF(AND(F39="نعم",G39="نعم"),"جرد + مراجعة",IF(F39="نعم","جرد فقط",IF(G39="نعم","مراجعة فقط",""))))</f>
         <v/>

</xml_diff>

<commit_message>
Add Al-Hassan Al-Ghunaimi to Sep 30 review of pharmacy 17
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -3364,7 +3364,11 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n"/>
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="B40" s="5">
         <f>IF(A40="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A40,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
@@ -3373,10 +3377,20 @@
         <f>IF(A40="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A40,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
         <v/>
       </c>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
+      <c r="D40" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H40" s="5">
         <f>IF(E40="","",IF(AND(F40="نعم",G40="نعم"),"جرد + مراجعة",IF(F40="نعم","جرد فقط",IF(G40="نعم","مراجعة فقط",""))))</f>
         <v/>

</xml_diff>

<commit_message>
Log Oct 1 count and reviews (pharmacy 28)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="C4" s="5">
         <f>IF(A4="","",COUNTIFS(السجل!$E$2:$E$1000,A4,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="5">
         <f>IF(A4="","",COUNTIFS(السجل!$E$2:$E$1000,A4,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -600,11 +600,11 @@
       </c>
       <c r="E4" s="5">
         <f>IF(A4="","",SUM(B4:D4))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" s="6">
         <f>IF(A4="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A4))</f>
-        <v>1800</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
       </c>
       <c r="C5" s="5">
         <f>IF(A5="","",COUNTIFS(السجل!$E$2:$E$1000,A5,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D5" s="5">
         <f>IF(A5="","",COUNTIFS(السجل!$E$2:$E$1000,A5,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -627,11 +627,11 @@
       </c>
       <c r="E5" s="5">
         <f>IF(A5="","",SUM(B5:D5))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" s="6">
         <f>IF(A5="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A5))</f>
-        <v>1500</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="6">
@@ -642,7 +642,7 @@
       </c>
       <c r="B6" s="5">
         <f>IF(A6="","",COUNTIFS(السجل!$E$2:$E$1000,A6,السجل!$H$2:$H$1000,"جرد + مراجعة"))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="5">
         <f>IF(A6="","",COUNTIFS(السجل!$E$2:$E$1000,A6,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
@@ -654,11 +654,11 @@
       </c>
       <c r="E6" s="5">
         <f>IF(A6="","",SUM(B6:D6))</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F6" s="6">
         <f>IF(A6="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A6))</f>
-        <v>1700</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="7">
@@ -673,7 +673,7 @@
       </c>
       <c r="C7" s="5">
         <f>IF(A7="","",COUNTIFS(السجل!$E$2:$E$1000,A7,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" s="5">
         <f>IF(A7="","",COUNTIFS(السجل!$E$2:$E$1000,A7,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -681,11 +681,11 @@
       </c>
       <c r="E7" s="5">
         <f>IF(A7="","",SUM(B7:D7))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F7" s="6">
         <f>IF(A7="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A7))</f>
-        <v>900</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="8">
@@ -700,7 +700,7 @@
       </c>
       <c r="C8" s="5">
         <f>IF(A8="","",COUNTIFS(السجل!$E$2:$E$1000,A8,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="5">
         <f>IF(A8="","",COUNTIFS(السجل!$E$2:$E$1000,A8,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -708,11 +708,11 @@
       </c>
       <c r="E8" s="5">
         <f>IF(A8="","",SUM(B8:D8))</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="6">
         <f>IF(A8="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A8))</f>
-        <v>450</v>
+        <v>600</v>
       </c>
     </row>
     <row r="9">
@@ -953,11 +953,11 @@
       </c>
       <c r="B19" s="7">
         <f>SUM(B4:B18)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C19" s="7">
         <f>SUM(C4:C18)</f>
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D19" s="7">
         <f>SUM(D4:D18)</f>
@@ -965,11 +965,11 @@
       </c>
       <c r="E19" s="7">
         <f>SUM(E4:E18)</f>
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F19" s="8">
         <f>SUM(F4:F18)</f>
-        <v>6350</v>
+        <v>7150</v>
       </c>
     </row>
     <row r="21">
@@ -980,7 +980,7 @@
       </c>
       <c r="F21" s="9">
         <f>SUM(السجل!$I$2:$I$1000)</f>
-        <v>6350</v>
+        <v>7150</v>
       </c>
     </row>
   </sheetData>
@@ -994,7 +994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1000"/>
+  <dimension ref="A1:H1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1003,7 +1003,8 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1044,6 +1045,12 @@
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
+          <t>الخميس
+2026-10-01</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
           <t>الإجمالي</t>
         </is>
       </c>
@@ -1073,9 +1080,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A2,السجل!$A$2:$A$1000,F$1000)</f>
         <v>400</v>
       </c>
-      <c r="G2" s="6">
-        <f>SUM(B2:F2)</f>
-        <v>1800</v>
+      <c r="G2" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A2,السجل!$A$2:$A$1000,G$1000)</f>
+        <v>150</v>
+      </c>
+      <c r="H2" s="6">
+        <f>SUM(B2:G2)</f>
+        <v>1950</v>
       </c>
     </row>
     <row r="3">
@@ -1103,9 +1114,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A3,السجل!$A$2:$A$1000,F$1000)</f>
         <v>300</v>
       </c>
-      <c r="G3" s="6">
-        <f>SUM(B3:F3)</f>
-        <v>1500</v>
+      <c r="G3" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A3,السجل!$A$2:$A$1000,G$1000)</f>
+        <v>150</v>
+      </c>
+      <c r="H3" s="6">
+        <f>SUM(B3:G3)</f>
+        <v>1650</v>
       </c>
     </row>
     <row r="4">
@@ -1133,9 +1148,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A4,السجل!$A$2:$A$1000,F$1000)</f>
         <v>300</v>
       </c>
-      <c r="G4" s="6">
-        <f>SUM(B4:F4)</f>
-        <v>1700</v>
+      <c r="G4" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A4,السجل!$A$2:$A$1000,G$1000)</f>
+        <v>200</v>
+      </c>
+      <c r="H4" s="6">
+        <f>SUM(B4:G4)</f>
+        <v>1900</v>
       </c>
     </row>
     <row r="5">
@@ -1163,9 +1182,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A5,السجل!$A$2:$A$1000,F$1000)</f>
         <v>300</v>
       </c>
-      <c r="G5" s="6">
-        <f>SUM(B5:F5)</f>
-        <v>900</v>
+      <c r="G5" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A5,السجل!$A$2:$A$1000,G$1000)</f>
+        <v>150</v>
+      </c>
+      <c r="H5" s="6">
+        <f>SUM(B5:G5)</f>
+        <v>1050</v>
       </c>
     </row>
     <row r="6">
@@ -1193,9 +1216,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A6,السجل!$A$2:$A$1000,F$1000)</f>
         <v>150</v>
       </c>
-      <c r="G6" s="6">
-        <f>SUM(B6:F6)</f>
-        <v>450</v>
+      <c r="G6" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A6,السجل!$A$2:$A$1000,G$1000)</f>
+        <v>150</v>
+      </c>
+      <c r="H6" s="6">
+        <f>SUM(B6:G6)</f>
+        <v>600</v>
       </c>
     </row>
     <row r="7">
@@ -1226,7 +1253,11 @@
       </c>
       <c r="G7" s="8">
         <f>SUM(G2:G6)</f>
-        <v>6350</v>
+        <v>800</v>
+      </c>
+      <c r="H7" s="8">
+        <f>SUM(H2:H6)</f>
+        <v>7150</v>
       </c>
     </row>
     <row r="1000" hidden="1">
@@ -1253,6 +1284,11 @@
       <c r="F1000" t="inlineStr">
         <is>
           <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -3678,118 +3714,192 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n"/>
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="B41" s="5" t="str">
         <f>IF(A41="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A41,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الخميس</v>
       </c>
       <c r="C41" s="5" t="str">
         <f>IF(A41="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A41,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H41" s="5" t="str">
         <f>IF(E41="","",IF(AND(F41="نعم",G41="نعم"),"جرد + مراجعة",IF(F41="نعم","جرد فقط",IF(G41="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I41" s="9">
         <f>IF(H41="جرد + مراجعة",الإعدادات!$B$2,IF(H41="مراجعة فقط",الإعدادات!$B$3,IF(H41="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n"/>
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="B42" s="5" t="str">
         <f>IF(A42="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A42,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الخميس</v>
       </c>
       <c r="C42" s="5" t="str">
         <f>IF(A42="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A42,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D42" s="4" t="n"/>
-      <c r="E42" s="4" t="n"/>
-      <c r="F42" s="4" t="n"/>
-      <c r="G42" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H42" s="5" t="str">
         <f>IF(E42="","",IF(AND(F42="نعم",G42="نعم"),"جرد + مراجعة",IF(F42="نعم","جرد فقط",IF(G42="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I42" s="9">
         <f>IF(H42="جرد + مراجعة",الإعدادات!$B$2,IF(H42="مراجعة فقط",الإعدادات!$B$3,IF(H42="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n"/>
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="B43" s="5" t="str">
         <f>IF(A43="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A43,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الخميس</v>
       </c>
       <c r="C43" s="5" t="str">
         <f>IF(A43="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A43,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H43" s="5" t="str">
         <f>IF(E43="","",IF(AND(F43="نعم",G43="نعم"),"جرد + مراجعة",IF(F43="نعم","جرد فقط",IF(G43="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I43" s="9">
         <f>IF(H43="جرد + مراجعة",الإعدادات!$B$2,IF(H43="مراجعة فقط",الإعدادات!$B$3,IF(H43="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="n"/>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="B44" s="5" t="str">
         <f>IF(A44="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A44,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الخميس</v>
       </c>
       <c r="C44" s="5" t="str">
         <f>IF(A44="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A44,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H44" s="5" t="str">
         <f>IF(E44="","",IF(AND(F44="نعم",G44="نعم"),"جرد + مراجعة",IF(F44="نعم","جرد فقط",IF(G44="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I44" s="9">
         <f>IF(H44="جرد + مراجعة",الإعدادات!$B$2,IF(H44="مراجعة فقط",الإعدادات!$B$3,IF(H44="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n"/>
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="B45" s="5" t="str">
         <f>IF(A45="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A45,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الخميس</v>
       </c>
       <c r="C45" s="5" t="str">
         <f>IF(A45="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A45,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H45" s="5" t="str">
         <f>IF(E45="","",IF(AND(F45="نعم",G45="نعم"),"جرد + مراجعة",IF(F45="نعم","جرد فقط",IF(G45="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I45" s="9">
         <f>IF(H45="جرد + مراجعة",الإعدادات!$B$2,IF(H45="مراجعة فقط",الإعدادات!$B$3,IF(H45="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="46">

</xml_diff>

<commit_message>
Log Oct 2 count and reviews (pharmacy 7)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="B4" s="5">
         <f>IF(A4="","",COUNTIFS(السجل!$E$2:$E$1000,A4,السجل!$H$2:$H$1000,"جرد + مراجعة"))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="5">
         <f>IF(A4="","",COUNTIFS(السجل!$E$2:$E$1000,A4,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
@@ -600,11 +600,11 @@
       </c>
       <c r="E4" s="5">
         <f>IF(A4="","",SUM(B4:D4))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4" s="6">
         <f>IF(A4="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A4))</f>
-        <v>1950</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
       </c>
       <c r="C5" s="5">
         <f>IF(A5="","",COUNTIFS(السجل!$E$2:$E$1000,A5,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="5">
         <f>IF(A5="","",COUNTIFS(السجل!$E$2:$E$1000,A5,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -627,11 +627,11 @@
       </c>
       <c r="E5" s="5">
         <f>IF(A5="","",SUM(B5:D5))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F5" s="6">
         <f>IF(A5="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A5))</f>
-        <v>1650</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="6">
@@ -646,7 +646,7 @@
       </c>
       <c r="C6" s="5">
         <f>IF(A6="","",COUNTIFS(السجل!$E$2:$E$1000,A6,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="5">
         <f>IF(A6="","",COUNTIFS(السجل!$E$2:$E$1000,A6,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -654,11 +654,11 @@
       </c>
       <c r="E6" s="5">
         <f>IF(A6="","",SUM(B6:D6))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F6" s="6">
         <f>IF(A6="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A6))</f>
-        <v>1900</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="7">
@@ -673,7 +673,7 @@
       </c>
       <c r="C7" s="5">
         <f>IF(A7="","",COUNTIFS(السجل!$E$2:$E$1000,A7,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" s="5">
         <f>IF(A7="","",COUNTIFS(السجل!$E$2:$E$1000,A7,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -681,11 +681,11 @@
       </c>
       <c r="E7" s="5">
         <f>IF(A7="","",SUM(B7:D7))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F7" s="6">
         <f>IF(A7="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A7))</f>
-        <v>1050</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8">
@@ -700,7 +700,7 @@
       </c>
       <c r="C8" s="5">
         <f>IF(A8="","",COUNTIFS(السجل!$E$2:$E$1000,A8,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="5">
         <f>IF(A8="","",COUNTIFS(السجل!$E$2:$E$1000,A8,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -708,11 +708,11 @@
       </c>
       <c r="E8" s="5">
         <f>IF(A8="","",SUM(B8:D8))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F8" s="6">
         <f>IF(A8="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A8))</f>
-        <v>600</v>
+        <v>750</v>
       </c>
     </row>
     <row r="9">
@@ -953,11 +953,11 @@
       </c>
       <c r="B19" s="7">
         <f>SUM(B4:B18)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C19" s="7">
         <f>SUM(C4:C18)</f>
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D19" s="7">
         <f>SUM(D4:D18)</f>
@@ -965,11 +965,11 @@
       </c>
       <c r="E19" s="7">
         <f>SUM(E4:E18)</f>
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="F19" s="8">
         <f>SUM(F4:F18)</f>
-        <v>7150</v>
+        <v>7950</v>
       </c>
     </row>
     <row r="21">
@@ -980,7 +980,7 @@
       </c>
       <c r="F21" s="9">
         <f>SUM(السجل!$I$2:$I$1000)</f>
-        <v>7150</v>
+        <v>7950</v>
       </c>
     </row>
   </sheetData>
@@ -994,7 +994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1000"/>
+  <dimension ref="A1:I1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1004,7 +1004,8 @@
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1051,6 +1052,12 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
+          <t>الجمعة
+2026-10-02</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>الإجمالي</t>
         </is>
       </c>
@@ -1084,9 +1091,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A2,السجل!$A$2:$A$1000,G$1000)</f>
         <v>150</v>
       </c>
-      <c r="H2" s="6">
-        <f>SUM(B2:G2)</f>
-        <v>1950</v>
+      <c r="H2" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A2,السجل!$A$2:$A$1000,H$1000)</f>
+        <v>200</v>
+      </c>
+      <c r="I2" s="6">
+        <f>SUM(B2:H2)</f>
+        <v>2150</v>
       </c>
     </row>
     <row r="3">
@@ -1118,9 +1129,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A3,السجل!$A$2:$A$1000,G$1000)</f>
         <v>150</v>
       </c>
-      <c r="H3" s="6">
-        <f>SUM(B3:G3)</f>
-        <v>1650</v>
+      <c r="H3" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A3,السجل!$A$2:$A$1000,H$1000)</f>
+        <v>150</v>
+      </c>
+      <c r="I3" s="6">
+        <f>SUM(B3:H3)</f>
+        <v>1800</v>
       </c>
     </row>
     <row r="4">
@@ -1152,9 +1167,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A4,السجل!$A$2:$A$1000,G$1000)</f>
         <v>200</v>
       </c>
-      <c r="H4" s="6">
-        <f>SUM(B4:G4)</f>
-        <v>1900</v>
+      <c r="H4" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A4,السجل!$A$2:$A$1000,H$1000)</f>
+        <v>150</v>
+      </c>
+      <c r="I4" s="6">
+        <f>SUM(B4:H4)</f>
+        <v>2050</v>
       </c>
     </row>
     <row r="5">
@@ -1186,9 +1205,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A5,السجل!$A$2:$A$1000,G$1000)</f>
         <v>150</v>
       </c>
-      <c r="H5" s="6">
-        <f>SUM(B5:G5)</f>
-        <v>1050</v>
+      <c r="H5" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A5,السجل!$A$2:$A$1000,H$1000)</f>
+        <v>150</v>
+      </c>
+      <c r="I5" s="6">
+        <f>SUM(B5:H5)</f>
+        <v>1200</v>
       </c>
     </row>
     <row r="6">
@@ -1220,9 +1243,13 @@
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A6,السجل!$A$2:$A$1000,G$1000)</f>
         <v>150</v>
       </c>
-      <c r="H6" s="6">
-        <f>SUM(B6:G6)</f>
-        <v>600</v>
+      <c r="H6" s="9">
+        <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A6,السجل!$A$2:$A$1000,H$1000)</f>
+        <v>150</v>
+      </c>
+      <c r="I6" s="6">
+        <f>SUM(B6:H6)</f>
+        <v>750</v>
       </c>
     </row>
     <row r="7">
@@ -1257,7 +1284,11 @@
       </c>
       <c r="H7" s="8">
         <f>SUM(H2:H6)</f>
-        <v>7150</v>
+        <v>800</v>
+      </c>
+      <c r="I7" s="8">
+        <f>SUM(I2:I6)</f>
+        <v>7950</v>
       </c>
     </row>
     <row r="1000" hidden="1">
@@ -1289,6 +1320,11 @@
       <c r="G1000" t="inlineStr">
         <is>
           <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -3903,118 +3939,192 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n"/>
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="B46" s="5" t="str">
         <f>IF(A46="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A46,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الجمعة</v>
       </c>
       <c r="C46" s="5" t="str">
         <f>IF(A46="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A46,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H46" s="5" t="str">
         <f>IF(E46="","",IF(AND(F46="نعم",G46="نعم"),"جرد + مراجعة",IF(F46="نعم","جرد فقط",IF(G46="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I46" s="9">
         <f>IF(H46="جرد + مراجعة",الإعدادات!$B$2,IF(H46="مراجعة فقط",الإعدادات!$B$3,IF(H46="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="n"/>
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="B47" s="5" t="str">
         <f>IF(A47="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A47,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الجمعة</v>
       </c>
       <c r="C47" s="5" t="str">
         <f>IF(A47="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A47,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H47" s="5" t="str">
         <f>IF(E47="","",IF(AND(F47="نعم",G47="نعم"),"جرد + مراجعة",IF(F47="نعم","جرد فقط",IF(G47="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I47" s="9">
         <f>IF(H47="جرد + مراجعة",الإعدادات!$B$2,IF(H47="مراجعة فقط",الإعدادات!$B$3,IF(H47="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n"/>
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="B48" s="5" t="str">
         <f>IF(A48="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A48,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الجمعة</v>
       </c>
       <c r="C48" s="5" t="str">
         <f>IF(A48="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A48,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H48" s="5" t="str">
         <f>IF(E48="","",IF(AND(F48="نعم",G48="نعم"),"جرد + مراجعة",IF(F48="نعم","جرد فقط",IF(G48="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I48" s="9">
         <f>IF(H48="جرد + مراجعة",الإعدادات!$B$2,IF(H48="مراجعة فقط",الإعدادات!$B$3,IF(H48="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="n"/>
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="B49" s="5" t="str">
         <f>IF(A49="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A49,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الجمعة</v>
       </c>
       <c r="C49" s="5" t="str">
         <f>IF(A49="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A49,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>د. أيمن حسين</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H49" s="5" t="str">
         <f>IF(E49="","",IF(AND(F49="نعم",G49="نعم"),"جرد + مراجعة",IF(F49="نعم","جرد فقط",IF(G49="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I49" s="9">
         <f>IF(H49="جرد + مراجعة",الإعدادات!$B$2,IF(H49="مراجعة فقط",الإعدادات!$B$3,IF(H49="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n"/>
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="B50" s="5" t="str">
         <f>IF(A50="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$28,MATCH(A50,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
+        <v>الجمعة</v>
       </c>
       <c r="C50" s="5" t="str">
         <f>IF(A50="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$28,MATCH(A50,'جدول الجرد'!$B$2:$B$28,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="4" t="n"/>
+        <v>الدلم</v>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="H50" s="5" t="str">
         <f>IF(E50="","",IF(AND(F50="نعم",G50="نعم"),"جرد + مراجعة",IF(F50="نعم","جرد فقط",IF(G50="نعم","مراجعة فقط",""))))</f>
-        <v/>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I50" s="9">
         <f>IF(H50="جرد + مراجعة",الإعدادات!$B$2,IF(H50="مراجعة فقط",الإعدادات!$B$3,IF(H50="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>0</v>
+        <v>150</v>
       </c>
     </row>
     <row r="51">

</xml_diff>

<commit_message>
Remove Mohamed Gamal from Oct 13 reviews; add Ayman Hussein to pharmacy 18 review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RnF4y3zxCG7NcjFkMnYdwu
</commit_message>
<xml_diff>
--- a/inventory/jard_payroll.xlsx
+++ b/inventory/jard_payroll.xlsx
@@ -646,7 +646,7 @@
       </c>
       <c r="C6" s="5">
         <f>IF(A6="","",COUNTIFS(السجل!$E$2:$E$1000,A6,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" s="5">
         <f>IF(A6="","",COUNTIFS(السجل!$E$2:$E$1000,A6,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -654,11 +654,11 @@
       </c>
       <c r="E6" s="5">
         <f>IF(A6="","",SUM(B6:D6))</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F6" s="6">
         <f>IF(A6="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A6))</f>
-        <v>1650</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
       </c>
       <c r="C9" s="5">
         <f>IF(A9="","",COUNTIFS(السجل!$E$2:$E$1000,A9,السجل!$H$2:$H$1000,"مراجعة فقط"))</f>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D9" s="5">
         <f>IF(A9="","",COUNTIFS(السجل!$E$2:$E$1000,A9,السجل!$H$2:$H$1000,"جرد فقط"))</f>
@@ -735,11 +735,11 @@
       </c>
       <c r="E9" s="5">
         <f>IF(A9="","",SUM(B9:D9))</f>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F9" s="6">
         <f>IF(A9="","",SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,A9))</f>
-        <v>2700</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="10">
@@ -965,7 +965,7 @@
       </c>
       <c r="C19" s="7">
         <f>SUM(C4:C18)</f>
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D19" s="7">
         <f>SUM(D4:D18)</f>
@@ -973,11 +973,11 @@
       </c>
       <c r="E19" s="7">
         <f>SUM(E4:E18)</f>
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F19" s="8">
         <f>SUM(F4:F18)</f>
-        <v>28800</v>
+        <v>28650</v>
       </c>
     </row>
     <row r="21">
@@ -988,7 +988,7 @@
       </c>
       <c r="F21" s="9">
         <f>SUM(السجل!$I$2:$I$1000)</f>
-        <v>28800</v>
+        <v>28650</v>
       </c>
     </row>
   </sheetData>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="W4" s="9">
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A4,السجل!$A$2:$A$1000,W$1000)</f>
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="X4" s="9">
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A4,السجل!$A$2:$A$1000,X$1000)</f>
@@ -1580,7 +1580,7 @@
       </c>
       <c r="AD4" s="6">
         <f>SUM(B4:AC4)</f>
-        <v>1650</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="5">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="T7" s="9">
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A7,السجل!$A$2:$A$1000,T$1000)</f>
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="U7" s="9">
         <f>SUMIFS(السجل!$I$2:$I$1000,السجل!$E$2:$E$1000,$A7,السجل!$A$2:$A$1000,U$1000)</f>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="AD7" s="6">
         <f>SUM(B7:AC7)</f>
-        <v>2700</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="8">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="T9" s="8">
         <f>SUM(T2:T8)</f>
-        <v>1300</v>
+        <v>1000</v>
       </c>
       <c r="U9" s="8">
         <f>SUM(U2:U8)</f>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="W9" s="8">
         <f>SUM(W2:W8)</f>
-        <v>650</v>
+        <v>800</v>
       </c>
       <c r="X9" s="8">
         <f>SUM(X2:X8)</f>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="AD9" s="8">
         <f>SUM(AD2:AD8)</f>
-        <v>28800</v>
+        <v>28650</v>
       </c>
     </row>
     <row r="1000" hidden="1">
@@ -8201,7 +8201,7 @@
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>د. محمد جمال</t>
+          <t>د. حسام شلش</t>
         </is>
       </c>
       <c r="F129" s="4" t="inlineStr"/>
@@ -8234,14 +8234,18 @@
         <v>الخرج</v>
       </c>
       <c r="D130" s="4" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F130" s="4" t="inlineStr"/>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G130" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8249,11 +8253,11 @@
       </c>
       <c r="H130" s="5" t="str">
         <f>IF(E130="","",IF(AND(F130="نعم",G130="نعم"),"جرد + مراجعة",IF(F130="نعم","جرد فقط",IF(G130="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I130" s="9">
         <f>IF(H130="جرد + مراجعة",الإعدادات!$B$2,IF(H130="مراجعة فقط",الإعدادات!$B$3,IF(H130="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="131">
@@ -8275,14 +8279,10 @@
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F131" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="inlineStr"/>
       <c r="G131" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8290,11 +8290,11 @@
       </c>
       <c r="H131" s="5" t="str">
         <f>IF(E131="","",IF(AND(F131="نعم",G131="نعم"),"جرد + مراجعة",IF(F131="نعم","جرد فقط",IF(G131="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I131" s="9">
         <f>IF(H131="جرد + مراجعة",الإعدادات!$B$2,IF(H131="مراجعة فقط",الإعدادات!$B$3,IF(H131="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="132">
@@ -8316,7 +8316,7 @@
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
+          <t>د. حسام شلش</t>
         </is>
       </c>
       <c r="F132" s="4" t="inlineStr"/>
@@ -8337,26 +8337,30 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B133" s="5" t="str">
         <f>IF(A133="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A133,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الثلاثاء</v>
+        <v>الأربعاء</v>
       </c>
       <c r="C133" s="5" t="str">
         <f>IF(A133="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A133,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الخرج</v>
       </c>
       <c r="D133" s="4" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>د. محمد جمال</t>
-        </is>
-      </c>
-      <c r="F133" s="4" t="inlineStr"/>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G133" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8364,33 +8368,33 @@
       </c>
       <c r="H133" s="5" t="str">
         <f>IF(E133="","",IF(AND(F133="نعم",G133="نعم"),"جرد + مراجعة",IF(F133="نعم","جرد فقط",IF(G133="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I133" s="9">
         <f>IF(H133="جرد + مراجعة",الإعدادات!$B$2,IF(H133="مراجعة فقط",الإعدادات!$B$3,IF(H133="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B134" s="5" t="str">
         <f>IF(A134="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A134,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الثلاثاء</v>
+        <v>الأربعاء</v>
       </c>
       <c r="C134" s="5" t="str">
         <f>IF(A134="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A134,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الخرج</v>
       </c>
       <c r="D134" s="4" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
+          <t>د. علي خليفة</t>
         </is>
       </c>
       <c r="F134" s="4" t="inlineStr"/>
@@ -8427,14 +8431,10 @@
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F135" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="inlineStr"/>
       <c r="G135" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8442,11 +8442,11 @@
       </c>
       <c r="H135" s="5" t="str">
         <f>IF(E135="","",IF(AND(F135="نعم",G135="نعم"),"جرد + مراجعة",IF(F135="نعم","جرد فقط",IF(G135="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I135" s="9">
         <f>IF(H135="جرد + مراجعة",الإعدادات!$B$2,IF(H135="مراجعة فقط",الإعدادات!$B$3,IF(H135="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="136">
@@ -8464,14 +8464,18 @@
         <v>الخرج</v>
       </c>
       <c r="D136" s="4" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F136" s="4" t="inlineStr"/>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G136" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8479,11 +8483,11 @@
       </c>
       <c r="H136" s="5" t="str">
         <f>IF(E136="","",IF(AND(F136="نعم",G136="نعم"),"جرد + مراجعة",IF(F136="نعم","جرد فقط",IF(G136="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I136" s="9">
         <f>IF(H136="جرد + مراجعة",الإعدادات!$B$2,IF(H136="مراجعة فقط",الإعدادات!$B$3,IF(H136="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="137">
@@ -8501,11 +8505,11 @@
         <v>الخرج</v>
       </c>
       <c r="D137" s="4" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
+          <t>د. علي خليفة</t>
         </is>
       </c>
       <c r="F137" s="4" t="inlineStr"/>
@@ -8542,14 +8546,10 @@
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F138" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="inlineStr"/>
       <c r="G138" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8557,36 +8557,40 @@
       </c>
       <c r="H138" s="5" t="str">
         <f>IF(E138="","",IF(AND(F138="نعم",G138="نعم"),"جرد + مراجعة",IF(F138="نعم","جرد فقط",IF(G138="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I138" s="9">
         <f>IF(H138="جرد + مراجعة",الإعدادات!$B$2,IF(H138="مراجعة فقط",الإعدادات!$B$3,IF(H138="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B139" s="5" t="str">
         <f>IF(A139="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A139,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الأربعاء</v>
+        <v>الخميس</v>
       </c>
       <c r="C139" s="5" t="str">
         <f>IF(A139="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A139,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الخرج</v>
       </c>
       <c r="D139" s="4" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
           <t>د. علي خليفة</t>
         </is>
       </c>
-      <c r="F139" s="4" t="inlineStr"/>
+      <c r="F139" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G139" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8594,33 +8598,33 @@
       </c>
       <c r="H139" s="5" t="str">
         <f>IF(E139="","",IF(AND(F139="نعم",G139="نعم"),"جرد + مراجعة",IF(F139="نعم","جرد فقط",IF(G139="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I139" s="9">
         <f>IF(H139="جرد + مراجعة",الإعدادات!$B$2,IF(H139="مراجعة فقط",الإعدادات!$B$3,IF(H139="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B140" s="5" t="str">
         <f>IF(A140="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A140,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الأربعاء</v>
+        <v>الخميس</v>
       </c>
       <c r="C140" s="5" t="str">
         <f>IF(A140="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A140,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الخرج</v>
       </c>
       <c r="D140" s="4" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
+          <t>د. حسام شلش</t>
         </is>
       </c>
       <c r="F140" s="4" t="inlineStr"/>
@@ -8657,14 +8661,10 @@
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F141" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F141" s="4" t="inlineStr"/>
       <c r="G141" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8672,11 +8672,11 @@
       </c>
       <c r="H141" s="5" t="str">
         <f>IF(E141="","",IF(AND(F141="نعم",G141="نعم"),"جرد + مراجعة",IF(F141="نعم","جرد فقط",IF(G141="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I141" s="9">
         <f>IF(H141="جرد + مراجعة",الإعدادات!$B$2,IF(H141="مراجعة فقط",الإعدادات!$B$3,IF(H141="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="142">
@@ -8694,14 +8694,18 @@
         <v>الخرج</v>
       </c>
       <c r="D142" s="4" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F142" s="4" t="inlineStr"/>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F142" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G142" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8709,11 +8713,11 @@
       </c>
       <c r="H142" s="5" t="str">
         <f>IF(E142="","",IF(AND(F142="نعم",G142="نعم"),"جرد + مراجعة",IF(F142="نعم","جرد فقط",IF(G142="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I142" s="9">
         <f>IF(H142="جرد + مراجعة",الإعدادات!$B$2,IF(H142="مراجعة فقط",الإعدادات!$B$3,IF(H142="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="143">
@@ -8731,11 +8735,11 @@
         <v>الخرج</v>
       </c>
       <c r="D143" s="4" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
+          <t>د. حسام شلش</t>
         </is>
       </c>
       <c r="F143" s="4" t="inlineStr"/>
@@ -8772,14 +8776,10 @@
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F144" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F144" s="4" t="inlineStr"/>
       <c r="G144" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8787,36 +8787,40 @@
       </c>
       <c r="H144" s="5" t="str">
         <f>IF(E144="","",IF(AND(F144="نعم",G144="نعم"),"جرد + مراجعة",IF(F144="نعم","جرد فقط",IF(G144="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I144" s="9">
         <f>IF(H144="جرد + مراجعة",الإعدادات!$B$2,IF(H144="مراجعة فقط",الإعدادات!$B$3,IF(H144="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B145" s="5" t="str">
         <f>IF(A145="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A145,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الخميس</v>
+        <v>الجمعة</v>
       </c>
       <c r="C145" s="5" t="str">
         <f>IF(A145="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A145,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الخرج</v>
       </c>
       <c r="D145" s="4" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
           <t>د. حسام شلش</t>
         </is>
       </c>
-      <c r="F145" s="4" t="inlineStr"/>
+      <c r="F145" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G145" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8824,33 +8828,33 @@
       </c>
       <c r="H145" s="5" t="str">
         <f>IF(E145="","",IF(AND(F145="نعم",G145="نعم"),"جرد + مراجعة",IF(F145="نعم","جرد فقط",IF(G145="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I145" s="9">
         <f>IF(H145="جرد + مراجعة",الإعدادات!$B$2,IF(H145="مراجعة فقط",الإعدادات!$B$3,IF(H145="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B146" s="5" t="str">
         <f>IF(A146="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A146,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الخميس</v>
+        <v>الجمعة</v>
       </c>
       <c r="C146" s="5" t="str">
         <f>IF(A146="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A146,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الخرج</v>
       </c>
       <c r="D146" s="4" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
+          <t>د. علي خليفة</t>
         </is>
       </c>
       <c r="F146" s="4" t="inlineStr"/>
@@ -8887,14 +8891,10 @@
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F147" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. الحسن الغنيمي</t>
+        </is>
+      </c>
+      <c r="F147" s="4" t="inlineStr"/>
       <c r="G147" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -8902,11 +8902,11 @@
       </c>
       <c r="H147" s="5" t="str">
         <f>IF(E147="","",IF(AND(F147="نعم",G147="نعم"),"جرد + مراجعة",IF(F147="نعم","جرد فقط",IF(G147="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I147" s="9">
         <f>IF(H147="جرد + مراجعة",الإعدادات!$B$2,IF(H147="مراجعة فقط",الإعدادات!$B$3,IF(H147="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="148">
@@ -8928,7 +8928,7 @@
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
+          <t>د. محمد فؤاد</t>
         </is>
       </c>
       <c r="F148" s="4" t="inlineStr"/>
@@ -8965,7 +8965,7 @@
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>د. الحسن الغنيمي</t>
+          <t>د. أيمن حسين</t>
         </is>
       </c>
       <c r="F149" s="4" t="inlineStr"/>
@@ -8986,26 +8986,30 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B150" s="5" t="str">
         <f>IF(A150="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A150,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الجمعة</v>
+        <v>السبت</v>
       </c>
       <c r="C150" s="5" t="str">
         <f>IF(A150="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A150,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الخرج</v>
       </c>
       <c r="D150" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>د. محمد فؤاد</t>
-        </is>
-      </c>
-      <c r="F150" s="4" t="inlineStr"/>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F150" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G150" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9013,11 +9017,11 @@
       </c>
       <c r="H150" s="5" t="str">
         <f>IF(E150="","",IF(AND(F150="نعم",G150="نعم"),"جرد + مراجعة",IF(F150="نعم","جرد فقط",IF(G150="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I150" s="9">
         <f>IF(H150="جرد + مراجعة",الإعدادات!$B$2,IF(H150="مراجعة فقط",الإعدادات!$B$3,IF(H150="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="151">
@@ -9039,14 +9043,10 @@
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F151" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F151" s="4" t="inlineStr"/>
       <c r="G151" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9054,11 +9054,11 @@
       </c>
       <c r="H151" s="5" t="str">
         <f>IF(E151="","",IF(AND(F151="نعم",G151="نعم"),"جرد + مراجعة",IF(F151="نعم","جرد فقط",IF(G151="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I151" s="9">
         <f>IF(H151="جرد + مراجعة",الإعدادات!$B$2,IF(H151="مراجعة فقط",الإعدادات!$B$3,IF(H151="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="152">
@@ -9080,7 +9080,7 @@
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
+          <t>د. حسام شلش</t>
         </is>
       </c>
       <c r="F152" s="4" t="inlineStr"/>
@@ -9101,26 +9101,30 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B153" s="5" t="str">
         <f>IF(A153="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A153,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>السبت</v>
+        <v>الأحد</v>
       </c>
       <c r="C153" s="5" t="str">
         <f>IF(A153="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A153,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الخرج</v>
       </c>
       <c r="D153" s="4" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
           <t>د. حسام شلش</t>
         </is>
       </c>
-      <c r="F153" s="4" t="inlineStr"/>
+      <c r="F153" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G153" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9128,11 +9132,11 @@
       </c>
       <c r="H153" s="5" t="str">
         <f>IF(E153="","",IF(AND(F153="نعم",G153="نعم"),"جرد + مراجعة",IF(F153="نعم","جرد فقط",IF(G153="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I153" s="9">
         <f>IF(H153="جرد + مراجعة",الإعدادات!$B$2,IF(H153="مراجعة فقط",الإعدادات!$B$3,IF(H153="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="154">
@@ -9154,14 +9158,10 @@
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F154" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F154" s="4" t="inlineStr"/>
       <c r="G154" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9169,11 +9169,11 @@
       </c>
       <c r="H154" s="5" t="str">
         <f>IF(E154="","",IF(AND(F154="نعم",G154="نعم"),"جرد + مراجعة",IF(F154="نعم","جرد فقط",IF(G154="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I154" s="9">
         <f>IF(H154="جرد + مراجعة",الإعدادات!$B$2,IF(H154="مراجعة فقط",الإعدادات!$B$3,IF(H154="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="155">
@@ -9195,7 +9195,7 @@
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
+          <t>د. السيد حسن</t>
         </is>
       </c>
       <c r="F155" s="4" t="inlineStr"/>
@@ -9216,26 +9216,30 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B156" s="5" t="str">
         <f>IF(A156="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A156,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الأحد</v>
+        <v>الاثنين</v>
       </c>
       <c r="C156" s="5" t="str">
         <f>IF(A156="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A156,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الخرج</v>
+        <v>الرياض</v>
       </c>
       <c r="D156" s="4" t="n">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
-        </is>
-      </c>
-      <c r="F156" s="4" t="inlineStr"/>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F156" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G156" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9243,11 +9247,11 @@
       </c>
       <c r="H156" s="5" t="str">
         <f>IF(E156="","",IF(AND(F156="نعم",G156="نعم"),"جرد + مراجعة",IF(F156="نعم","جرد فقط",IF(G156="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I156" s="9">
         <f>IF(H156="جرد + مراجعة",الإعدادات!$B$2,IF(H156="مراجعة فقط",الإعدادات!$B$3,IF(H156="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="157">
@@ -9269,14 +9273,10 @@
       </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F157" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F157" s="4" t="inlineStr"/>
       <c r="G157" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9284,11 +9284,11 @@
       </c>
       <c r="H157" s="5" t="str">
         <f>IF(E157="","",IF(AND(F157="نعم",G157="نعم"),"جرد + مراجعة",IF(F157="نعم","جرد فقط",IF(G157="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I157" s="9">
         <f>IF(H157="جرد + مراجعة",الإعدادات!$B$2,IF(H157="مراجعة فقط",الإعدادات!$B$3,IF(H157="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="158">
@@ -9310,7 +9310,7 @@
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
+          <t>د. السيد حسن</t>
         </is>
       </c>
       <c r="F158" s="4" t="inlineStr"/>
@@ -9343,14 +9343,18 @@
         <v>الرياض</v>
       </c>
       <c r="D159" s="4" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
-        </is>
-      </c>
-      <c r="F159" s="4" t="inlineStr"/>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F159" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G159" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9358,11 +9362,11 @@
       </c>
       <c r="H159" s="5" t="str">
         <f>IF(E159="","",IF(AND(F159="نعم",G159="نعم"),"جرد + مراجعة",IF(F159="نعم","جرد فقط",IF(G159="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I159" s="9">
         <f>IF(H159="جرد + مراجعة",الإعدادات!$B$2,IF(H159="مراجعة فقط",الإعدادات!$B$3,IF(H159="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="160">
@@ -9384,14 +9388,10 @@
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F160" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F160" s="4" t="inlineStr"/>
       <c r="G160" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9399,11 +9399,11 @@
       </c>
       <c r="H160" s="5" t="str">
         <f>IF(E160="","",IF(AND(F160="نعم",G160="نعم"),"جرد + مراجعة",IF(F160="نعم","جرد فقط",IF(G160="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I160" s="9">
         <f>IF(H160="جرد + مراجعة",الإعدادات!$B$2,IF(H160="مراجعة فقط",الإعدادات!$B$3,IF(H160="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="161">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
+          <t>د. السيد حسن</t>
         </is>
       </c>
       <c r="F161" s="4" t="inlineStr"/>
@@ -9446,26 +9446,30 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B162" s="5" t="str">
         <f>IF(A162="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A162,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الاثنين</v>
+        <v>الثلاثاء</v>
       </c>
       <c r="C162" s="5" t="str">
         <f>IF(A162="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A162,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الرياض</v>
       </c>
       <c r="D162" s="4" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
-        </is>
-      </c>
-      <c r="F162" s="4" t="inlineStr"/>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G162" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9473,11 +9477,11 @@
       </c>
       <c r="H162" s="5" t="str">
         <f>IF(E162="","",IF(AND(F162="نعم",G162="نعم"),"جرد + مراجعة",IF(F162="نعم","جرد فقط",IF(G162="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I162" s="9">
         <f>IF(H162="جرد + مراجعة",الإعدادات!$B$2,IF(H162="مراجعة فقط",الإعدادات!$B$3,IF(H162="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="163">
@@ -9499,14 +9503,10 @@
       </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F163" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F163" s="4" t="inlineStr"/>
       <c r="G163" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9514,11 +9514,11 @@
       </c>
       <c r="H163" s="5" t="str">
         <f>IF(E163="","",IF(AND(F163="نعم",G163="نعم"),"جرد + مراجعة",IF(F163="نعم","جرد فقط",IF(G163="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I163" s="9">
         <f>IF(H163="جرد + مراجعة",الإعدادات!$B$2,IF(H163="مراجعة فقط",الإعدادات!$B$3,IF(H163="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="164">
@@ -9536,14 +9536,18 @@
         <v>الرياض</v>
       </c>
       <c r="D164" s="4" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
-        </is>
-      </c>
-      <c r="F164" s="4" t="inlineStr"/>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F164" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G164" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9551,11 +9555,11 @@
       </c>
       <c r="H164" s="5" t="str">
         <f>IF(E164="","",IF(AND(F164="نعم",G164="نعم"),"جرد + مراجعة",IF(F164="نعم","جرد فقط",IF(G164="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I164" s="9">
         <f>IF(H164="جرد + مراجعة",الإعدادات!$B$2,IF(H164="مراجعة فقط",الإعدادات!$B$3,IF(H164="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="165">
@@ -9577,14 +9581,10 @@
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F165" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F165" s="4" t="inlineStr"/>
       <c r="G165" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9592,36 +9592,40 @@
       </c>
       <c r="H165" s="5" t="str">
         <f>IF(E165="","",IF(AND(F165="نعم",G165="نعم"),"جرد + مراجعة",IF(F165="نعم","جرد فقط",IF(G165="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I165" s="9">
         <f>IF(H165="جرد + مراجعة",الإعدادات!$B$2,IF(H165="مراجعة فقط",الإعدادات!$B$3,IF(H165="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B166" s="5" t="str">
         <f>IF(A166="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A166,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الثلاثاء</v>
+        <v>الأربعاء</v>
       </c>
       <c r="C166" s="5" t="str">
         <f>IF(A166="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A166,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
         <v>الرياض</v>
       </c>
       <c r="D166" s="4" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
-        </is>
-      </c>
-      <c r="F166" s="4" t="inlineStr"/>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F166" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G166" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9629,11 +9633,11 @@
       </c>
       <c r="H166" s="5" t="str">
         <f>IF(E166="","",IF(AND(F166="نعم",G166="نعم"),"جرد + مراجعة",IF(F166="نعم","جرد فقط",IF(G166="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I166" s="9">
         <f>IF(H166="جرد + مراجعة",الإعدادات!$B$2,IF(H166="مراجعة فقط",الإعدادات!$B$3,IF(H166="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="167">
@@ -9655,14 +9659,10 @@
       </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F167" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F167" s="4" t="inlineStr"/>
       <c r="G167" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9670,11 +9670,11 @@
       </c>
       <c r="H167" s="5" t="str">
         <f>IF(E167="","",IF(AND(F167="نعم",G167="نعم"),"جرد + مراجعة",IF(F167="نعم","جرد فقط",IF(G167="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I167" s="9">
         <f>IF(H167="جرد + مراجعة",الإعدادات!$B$2,IF(H167="مراجعة فقط",الإعدادات!$B$3,IF(H167="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="168">
@@ -9696,7 +9696,7 @@
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
+          <t>د. السيد حسن</t>
         </is>
       </c>
       <c r="F168" s="4" t="inlineStr"/>
@@ -9729,14 +9729,18 @@
         <v>الرياض</v>
       </c>
       <c r="D169" s="4" t="n">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
-        </is>
-      </c>
-      <c r="F169" s="4" t="inlineStr"/>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F169" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G169" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9744,11 +9748,11 @@
       </c>
       <c r="H169" s="5" t="str">
         <f>IF(E169="","",IF(AND(F169="نعم",G169="نعم"),"جرد + مراجعة",IF(F169="نعم","جرد فقط",IF(G169="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I169" s="9">
         <f>IF(H169="جرد + مراجعة",الإعدادات!$B$2,IF(H169="مراجعة فقط",الإعدادات!$B$3,IF(H169="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="170">
@@ -9770,14 +9774,10 @@
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F170" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F170" s="4" t="inlineStr"/>
       <c r="G170" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9785,11 +9785,11 @@
       </c>
       <c r="H170" s="5" t="str">
         <f>IF(E170="","",IF(AND(F170="نعم",G170="نعم"),"جرد + مراجعة",IF(F170="نعم","جرد فقط",IF(G170="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I170" s="9">
         <f>IF(H170="جرد + مراجعة",الإعدادات!$B$2,IF(H170="مراجعة فقط",الإعدادات!$B$3,IF(H170="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="171">
@@ -9811,7 +9811,7 @@
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
+          <t>د. السيد حسن</t>
         </is>
       </c>
       <c r="F171" s="4" t="inlineStr"/>
@@ -9832,26 +9832,30 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B172" s="5" t="str">
         <f>IF(A172="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A172,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الأربعاء</v>
+        <v>الخميس</v>
       </c>
       <c r="C172" s="5" t="str">
         <f>IF(A172="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A172,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الرياض</v>
+        <v>الخرج</v>
       </c>
       <c r="D172" s="4" t="n">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
-        </is>
-      </c>
-      <c r="F172" s="4" t="inlineStr"/>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F172" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G172" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9859,11 +9863,11 @@
       </c>
       <c r="H172" s="5" t="str">
         <f>IF(E172="","",IF(AND(F172="نعم",G172="نعم"),"جرد + مراجعة",IF(F172="نعم","جرد فقط",IF(G172="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I172" s="9">
         <f>IF(H172="جرد + مراجعة",الإعدادات!$B$2,IF(H172="مراجعة فقط",الإعدادات!$B$3,IF(H172="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="173">
@@ -9885,14 +9889,10 @@
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F173" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. علي خليفة</t>
+        </is>
+      </c>
+      <c r="F173" s="4" t="inlineStr"/>
       <c r="G173" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9900,11 +9900,11 @@
       </c>
       <c r="H173" s="5" t="str">
         <f>IF(E173="","",IF(AND(F173="نعم",G173="نعم"),"جرد + مراجعة",IF(F173="نعم","جرد فقط",IF(G173="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I173" s="9">
         <f>IF(H173="جرد + مراجعة",الإعدادات!$B$2,IF(H173="مراجعة فقط",الإعدادات!$B$3,IF(H173="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="174">
@@ -9922,14 +9922,18 @@
         <v>الخرج</v>
       </c>
       <c r="D174" s="4" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F174" s="4" t="inlineStr"/>
+          <t>د. حسام شلش</t>
+        </is>
+      </c>
+      <c r="F174" s="4" t="inlineStr">
+        <is>
+          <t>نعم</t>
+        </is>
+      </c>
       <c r="G174" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9937,11 +9941,11 @@
       </c>
       <c r="H174" s="5" t="str">
         <f>IF(E174="","",IF(AND(F174="نعم",G174="نعم"),"جرد + مراجعة",IF(F174="نعم","جرد فقط",IF(G174="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v>جرد + مراجعة</v>
       </c>
       <c r="I174" s="9">
         <f>IF(H174="جرد + مراجعة",الإعدادات!$B$2,IF(H174="مراجعة فقط",الإعدادات!$B$3,IF(H174="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>200</v>
       </c>
     </row>
     <row r="175">
@@ -9963,14 +9967,10 @@
       </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
-          <t>د. حسام شلش</t>
-        </is>
-      </c>
-      <c r="F175" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+          <t>د. السيد حسن</t>
+        </is>
+      </c>
+      <c r="F175" s="4" t="inlineStr"/>
       <c r="G175" s="4" t="inlineStr">
         <is>
           <t>نعم</t>
@@ -9978,11 +9978,11 @@
       </c>
       <c r="H175" s="5" t="str">
         <f>IF(E175="","",IF(AND(F175="نعم",G175="نعم"),"جرد + مراجعة",IF(F175="نعم","جرد فقط",IF(G175="نعم","مراجعة فقط",""))))</f>
-        <v>جرد + مراجعة</v>
+        <v>مراجعة فقط</v>
       </c>
       <c r="I175" s="9">
         <f>IF(H175="جرد + مراجعة",الإعدادات!$B$2,IF(H175="مراجعة فقط",الإعدادات!$B$3,IF(H175="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="176">
@@ -10004,7 +10004,7 @@
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>د. السيد حسن</t>
+          <t>د. علي خليفة</t>
         </is>
       </c>
       <c r="F176" s="4" t="inlineStr"/>
@@ -10023,40 +10023,26 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
+      <c r="A177" s="4" t="n"/>
       <c r="B177" s="5" t="str">
         <f>IF(A177="","",IFERROR(INDEX('جدول الجرد'!$A$2:$A$31,MATCH(A177,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الخميس</v>
+        <v/>
       </c>
       <c r="C177" s="5" t="str">
         <f>IF(A177="","",IFERROR(INDEX('جدول الجرد'!$E$2:$E$31,MATCH(A177,'جدول الجرد'!$B$2:$B$31,0)),""))</f>
-        <v>الخرج</v>
-      </c>
-      <c r="D177" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="E177" s="4" t="inlineStr">
-        <is>
-          <t>د. علي خليفة</t>
-        </is>
-      </c>
-      <c r="F177" s="4" t="inlineStr"/>
-      <c r="G177" s="4" t="inlineStr">
-        <is>
-          <t>نعم</t>
-        </is>
-      </c>
+        <v/>
+      </c>
+      <c r="D177" s="4" t="n"/>
+      <c r="E177" s="4" t="n"/>
+      <c r="F177" s="4" t="n"/>
+      <c r="G177" s="4" t="n"/>
       <c r="H177" s="5" t="str">
         <f>IF(E177="","",IF(AND(F177="نعم",G177="نعم"),"جرد + مراجعة",IF(F177="نعم","جرد فقط",IF(G177="نعم","مراجعة فقط",""))))</f>
-        <v>مراجعة فقط</v>
+        <v/>
       </c>
       <c r="I177" s="9">
         <f>IF(H177="جرد + مراجعة",الإعدادات!$B$2,IF(H177="مراجعة فقط",الإعدادات!$B$3,IF(H177="جرد فقط",الإعدادات!$B$4,0)))</f>
-        <v>150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178">

</xml_diff>